<commit_message>
Fix arid_humans data-quality issues from ARID_inconsistencias_datos.xlsx review
- Rotate sample_type/element/tissue_type for 692 rows from a mis-mapped
  import batch (Knudson & Torres 2023, Pestle et al. 2021, Standen et al.
  2025)
- Add 32 Peru sites (arid_sites) referenced by arid_humans but missing,
  derived from existing lat/lon/period data
- Unify sex vocabulary to F/M/Indeterminate
- Fix "MIddle Adult" typo
- Convert has_c14 to logical; resolve 8 NA rows with no lab_id to FALSE
- Correct stale doc: sample_id is an individual identifier (not unique per
  row), lab_id only expected to match arid_c14 when has_c14=TRUE,
  arid_animals$type_source is Marine/Terrestrial fauna (not wild/domestic),
  document cross-reference duplicate sample_id, refresh stale row counts

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/data_xlsx/arid_sites.xlsx
+++ b/data/data_xlsx/arid_sites.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K438"/>
+  <dimension ref="A1:K470"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -15335,6 +15335,1510 @@
         </is>
       </c>
     </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Middle Osmore, Moquegua Basin</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Algodonal</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G439">
+        <v>1000</v>
+      </c>
+      <c r="H439">
+        <v>1470</v>
+      </c>
+      <c r="I439">
+        <v>-17.612697</v>
+      </c>
+      <c r="J439">
+        <v>-71.242814</v>
+      </c>
+      <c r="K439">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Chen Chen</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G440">
+        <v>850</v>
+      </c>
+      <c r="H440">
+        <v>1100</v>
+      </c>
+      <c r="I440">
+        <v>-17.194964</v>
+      </c>
+      <c r="J440">
+        <v>-70.919729</v>
+      </c>
+      <c r="K440">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Chiribaya Alta</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G441">
+        <v>1000</v>
+      </c>
+      <c r="H441">
+        <v>1470</v>
+      </c>
+      <c r="I441">
+        <v>-17.631102</v>
+      </c>
+      <c r="J441">
+        <v>-71.29707999999999</v>
+      </c>
+      <c r="K441">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Chiribaya Baja</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G442">
+        <v>1000</v>
+      </c>
+      <c r="H442">
+        <v>1470</v>
+      </c>
+      <c r="I442">
+        <v>-17.6281</v>
+      </c>
+      <c r="J442">
+        <v>-71.2791</v>
+      </c>
+      <c r="K442">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Middle Osmore, Moquegua Basin</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Estuquina</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G443">
+        <v>1000</v>
+      </c>
+      <c r="H443">
+        <v>1470</v>
+      </c>
+      <c r="I443">
+        <v>-17.16</v>
+      </c>
+      <c r="J443">
+        <v>-70.92</v>
+      </c>
+      <c r="K443">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>La Cruz</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G444">
+        <v>850</v>
+      </c>
+      <c r="H444">
+        <v>1100</v>
+      </c>
+      <c r="I444">
+        <v>-17.63</v>
+      </c>
+      <c r="J444">
+        <v>-71.28</v>
+      </c>
+      <c r="K444">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>La Victoria</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G445">
+        <v>850</v>
+      </c>
+      <c r="H445">
+        <v>1100</v>
+      </c>
+      <c r="I445">
+        <v>-17.63</v>
+      </c>
+      <c r="J445">
+        <v>-71.28</v>
+      </c>
+      <c r="K445">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>North to Ilo city, Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Roca Verde</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="G446">
+        <v>-500</v>
+      </c>
+      <c r="H446">
+        <v>200</v>
+      </c>
+      <c r="I446">
+        <v>-17.54</v>
+      </c>
+      <c r="J446">
+        <v>-71.36</v>
+      </c>
+      <c r="K446">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>North to Ilo city, Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Wakaki</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="G447">
+        <v>340</v>
+      </c>
+      <c r="H447">
+        <v>340</v>
+      </c>
+      <c r="I447">
+        <v>-17.49</v>
+      </c>
+      <c r="J447">
+        <v>-71.36</v>
+      </c>
+      <c r="K447">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>San Geronimo</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G448">
+        <v>1000</v>
+      </c>
+      <c r="H448">
+        <v>1470</v>
+      </c>
+      <c r="I448">
+        <v>-17.625638</v>
+      </c>
+      <c r="J448">
+        <v>-71.336865</v>
+      </c>
+      <c r="K448">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>El Yaral</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G449">
+        <v>1000</v>
+      </c>
+      <c r="H449">
+        <v>1200</v>
+      </c>
+      <c r="I449">
+        <v>-17.363927</v>
+      </c>
+      <c r="J449">
+        <v>-71.015711</v>
+      </c>
+      <c r="K449">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Chen Chen(B)</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G450">
+        <v>850</v>
+      </c>
+      <c r="H450">
+        <v>1100</v>
+      </c>
+      <c r="I450">
+        <v>-17.194964</v>
+      </c>
+      <c r="J450">
+        <v>-70.919729</v>
+      </c>
+      <c r="K450">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Chen Chen(C)</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G451">
+        <v>850</v>
+      </c>
+      <c r="H451">
+        <v>1100</v>
+      </c>
+      <c r="I451">
+        <v>-17.194964</v>
+      </c>
+      <c r="J451">
+        <v>-70.919729</v>
+      </c>
+      <c r="K451">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Chen Chen(L)</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G452">
+        <v>850</v>
+      </c>
+      <c r="H452">
+        <v>1100</v>
+      </c>
+      <c r="I452">
+        <v>-17.194964</v>
+      </c>
+      <c r="J452">
+        <v>-70.919729</v>
+      </c>
+      <c r="K452">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Chen Chen(A)</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G453">
+        <v>850</v>
+      </c>
+      <c r="H453">
+        <v>1100</v>
+      </c>
+      <c r="I453">
+        <v>-17.194964</v>
+      </c>
+      <c r="J453">
+        <v>-70.919729</v>
+      </c>
+      <c r="K453">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Chen Chen(I)</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G454">
+        <v>850</v>
+      </c>
+      <c r="H454">
+        <v>1100</v>
+      </c>
+      <c r="I454">
+        <v>-17.194964</v>
+      </c>
+      <c r="J454">
+        <v>-70.919729</v>
+      </c>
+      <c r="K454">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Chen Chen(K)</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G455">
+        <v>850</v>
+      </c>
+      <c r="H455">
+        <v>1100</v>
+      </c>
+      <c r="I455">
+        <v>-17.194964</v>
+      </c>
+      <c r="J455">
+        <v>-70.919729</v>
+      </c>
+      <c r="K455">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Chen Chen(D)</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G456">
+        <v>850</v>
+      </c>
+      <c r="H456">
+        <v>1100</v>
+      </c>
+      <c r="I456">
+        <v>-17.194964</v>
+      </c>
+      <c r="J456">
+        <v>-70.919729</v>
+      </c>
+      <c r="K456">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Chen Chen(E)</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G457">
+        <v>850</v>
+      </c>
+      <c r="H457">
+        <v>1100</v>
+      </c>
+      <c r="I457">
+        <v>-17.194964</v>
+      </c>
+      <c r="J457">
+        <v>-70.919729</v>
+      </c>
+      <c r="K457">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Chiribaya Alta(3)</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G458">
+        <v>1000</v>
+      </c>
+      <c r="H458">
+        <v>1470</v>
+      </c>
+      <c r="I458">
+        <v>-17.631102</v>
+      </c>
+      <c r="J458">
+        <v>-71.29707999999999</v>
+      </c>
+      <c r="K458">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Chiribaya Alta(4)</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G459">
+        <v>1000</v>
+      </c>
+      <c r="H459">
+        <v>1470</v>
+      </c>
+      <c r="I459">
+        <v>-17.631102</v>
+      </c>
+      <c r="J459">
+        <v>-71.29707999999999</v>
+      </c>
+      <c r="K459">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Chiribaya Alta(7)</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G460">
+        <v>1000</v>
+      </c>
+      <c r="H460">
+        <v>1470</v>
+      </c>
+      <c r="I460">
+        <v>-17.631102</v>
+      </c>
+      <c r="J460">
+        <v>-71.29707999999999</v>
+      </c>
+      <c r="K460">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Lower Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Coast</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Chiribaya Baja(1)</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G461">
+        <v>1000</v>
+      </c>
+      <c r="H461">
+        <v>1470</v>
+      </c>
+      <c r="I461">
+        <v>-17.6281</v>
+      </c>
+      <c r="J461">
+        <v>-71.2791</v>
+      </c>
+      <c r="K461">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Rio Muerto</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G462">
+        <v>500</v>
+      </c>
+      <c r="H462">
+        <v>1100</v>
+      </c>
+      <c r="I462">
+        <v>-17.173132</v>
+      </c>
+      <c r="J462">
+        <v>-70.98350000000001</v>
+      </c>
+      <c r="K462">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Loreto Viejo</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="G463">
+        <v>-100</v>
+      </c>
+      <c r="H463">
+        <v>350</v>
+      </c>
+      <c r="I463">
+        <v>-17.60261</v>
+      </c>
+      <c r="J463">
+        <v>-71.231786</v>
+      </c>
+      <c r="K463">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Omo</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Formative</t>
+        </is>
+      </c>
+      <c r="G464">
+        <v>1</v>
+      </c>
+      <c r="H464">
+        <v>150</v>
+      </c>
+      <c r="I464">
+        <v>-17.244</v>
+      </c>
+      <c r="J464">
+        <v>-70.9802</v>
+      </c>
+      <c r="K464">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Omo M10</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G465">
+        <v>785</v>
+      </c>
+      <c r="H465">
+        <v>1000</v>
+      </c>
+      <c r="I465">
+        <v>-17.244</v>
+      </c>
+      <c r="J465">
+        <v>-70.9802</v>
+      </c>
+      <c r="K465">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Rio Muerto M43</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G466">
+        <v>500</v>
+      </c>
+      <c r="H466">
+        <v>1100</v>
+      </c>
+      <c r="I466">
+        <v>-17.173132</v>
+      </c>
+      <c r="J466">
+        <v>-70.98350000000001</v>
+      </c>
+      <c r="K466">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Middle Osmore Valley</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Rio Muerto M70</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Middle Horizon</t>
+        </is>
+      </c>
+      <c r="G467">
+        <v>500</v>
+      </c>
+      <c r="H467">
+        <v>1100</v>
+      </c>
+      <c r="I467">
+        <v>-17.173132</v>
+      </c>
+      <c r="J467">
+        <v>-70.98350000000001</v>
+      </c>
+      <c r="K467">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Moquegua</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Middle Osmore, Moquegua Basin</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Precordillera</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Tumilaca La Chimba</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Late Intermediate (Estuquina phase)</t>
+        </is>
+      </c>
+      <c r="G468">
+        <v>950</v>
+      </c>
+      <c r="H468">
+        <v>1450</v>
+      </c>
+      <c r="I468">
+        <v>-17.1467</v>
+      </c>
+      <c r="J468">
+        <v>-70.8584</v>
+      </c>
+      <c r="K468">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Tacna</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Alto de la Alianza, Middle Valley of Tacna</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Alto de la Alianza</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Modern</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="G469">
+        <v>1850</v>
+      </c>
+      <c r="H469">
+        <v>1880</v>
+      </c>
+      <c r="I469">
+        <v>-18.008121</v>
+      </c>
+      <c r="J469">
+        <v>-70.313366</v>
+      </c>
+      <c r="K469">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Tacna</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Lower Sama Valley, Sama Grande</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Lowlands</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Los Batanes</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Late Intermediate</t>
+        </is>
+      </c>
+      <c r="G470">
+        <v>1000</v>
+      </c>
+      <c r="H470">
+        <v>1100</v>
+      </c>
+      <c r="I470">
+        <v>-17.815633</v>
+      </c>
+      <c r="J470">
+        <v>-70.511501</v>
+      </c>
+      <c r="K470">
+        <v>506</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix ecozone: Antofagasta oasis sites mislabeled Altiplano -> Precordillera
630 arid_humans rows at San Pedro de Atacama oasis sites (Coyo, Solcor,
Quitor, Tchecar, Catarpe, Larache, Casa Parroquial, Solor Villama, Yaye)
had ecozone incorrectly set to Altiplano under Pestle et al. (2021) and
Knudson and Torres (2023), while every other reference at the same sites
correctly used Precordillera. arid_sites corrected to match for the 5
sites with no other reference to confirm against.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/data_xlsx/arid_sites.xlsx
+++ b/data/data_xlsx/arid_sites.xlsx
@@ -14874,7 +14874,7 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Altiplano</t>
+          <t>Precordillera</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Altiplano</t>
+          <t>Precordillera</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Altiplano</t>
+          <t>Precordillera</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
@@ -15095,7 +15095,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Altiplano</t>
+          <t>Precordillera</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Altiplano</t>
+          <t>Precordillera</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">

</xml_diff>